<commit_message>
Refactor/Removing faulty evaluation results
</commit_message>
<xml_diff>
--- a/src/evaluation/data/scraping_stats_Naive.xlsx
+++ b/src/evaluation/data/scraping_stats_Naive.xlsx
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>12.62</v>
+        <v>12.41</v>
       </c>
     </row>
     <row r="15">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>757</v>
+        <v>744</v>
       </c>
     </row>
     <row r="16">
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3.53</v>
+        <v>3.59</v>
       </c>
     </row>
     <row r="17">
@@ -602,7 +602,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2025-12-11 15:12:42</t>
+          <t>2025-12-17 10:48:03</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2025-12-11 15:25:20</t>
+          <t>2025-12-17 11:00:27</t>
         </is>
       </c>
     </row>

</xml_diff>